<commit_message>
Corrections description suite review NRISS 4bf4611faff0252f2825ea8b2af2f0b3207bfed1
</commit_message>
<xml_diff>
--- a/URLCanonique/ig/StructureDefinition-FRLMAttachments.xlsx
+++ b/URLCanonique/ig/StructureDefinition-FRLMAttachments.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-30T08:39:54+00:00</t>
+    <t>2026-09-30T08:56:57+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -375,7 +375,7 @@
 </t>
   </si>
   <si>
-    <t>Simple observation : Permet d'indiquer la nature des documents ajoutés</t>
+    <t>Permet d'indiquer la nature des documents ajoutés</t>
   </si>
   <si>
     <t>FRLMAttachments.entry.attachment</t>

</xml_diff>